<commit_message>
Switch column naming and row naming to prevent overwriting column name "Mask"
</commit_message>
<xml_diff>
--- a/output/remaining_area_and_pixels.xlsx
+++ b/output/remaining_area_and_pixels.xlsx
@@ -375,7 +375,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Mask</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Mask</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Mask</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Mask</t>
         </is>
       </c>
     </row>

</xml_diff>